<commit_message>
feat: add Plan Görünümü (clipping plane mode) to scene 4
- Add toggle-2 clip mode: orthographic camera, 45° angle, 50% clipping plane
- Add 6 room hotspots with name + m² labels visible in clip mode
- Restructure Excel: room buttons use toggle-1, panels keyed by button ID (cam1-left etc.)
- Support multi-line hotspot labels (\n splits into name + gold m² line)
- Switch between perspective (room tour) and orthographic (plan view) cameras
- Auto-restore materials and camera when exiting clip mode

https://claude.ai/code/session_01NbLjFLHf9cNBKyb3QMv6fy
</commit_message>
<xml_diff>
--- a/demo2-xlsx/demo2-input_4.xlsx
+++ b/demo2-xlsx/demo2-input_4.xlsx
@@ -26466,7 +26466,7 @@
       </c>
       <c r="E520" s="19" t="inlineStr">
         <is>
-          <t>toggle-2</t>
+          <t>toggle-1</t>
         </is>
       </c>
       <c r="F520" s="19" t="n"/>
@@ -26501,7 +26501,7 @@
       </c>
       <c r="E521" s="19" t="inlineStr">
         <is>
-          <t>toggle-3</t>
+          <t>toggle-1</t>
         </is>
       </c>
       <c r="F521" s="19" t="n"/>
@@ -26536,7 +26536,7 @@
       </c>
       <c r="E522" s="19" t="inlineStr">
         <is>
-          <t>toggle-4</t>
+          <t>toggle-1</t>
         </is>
       </c>
       <c r="F522" s="19" t="n"/>
@@ -26571,7 +26571,7 @@
       </c>
       <c r="E523" s="19" t="inlineStr">
         <is>
-          <t>toggle-5</t>
+          <t>toggle-1</t>
         </is>
       </c>
       <c r="F523" s="19" t="n"/>
@@ -26606,7 +26606,7 @@
       </c>
       <c r="E524" s="19" t="inlineStr">
         <is>
-          <t>toggle-6</t>
+          <t>toggle-1</t>
         </is>
       </c>
       <c r="F524" s="19" t="n"/>
@@ -26621,29 +26621,27 @@
       <c r="O524" s="19" t="n"/>
     </row>
     <row r="525">
-      <c r="A525" s="21" t="inlineStr">
-        <is>
-          <t>slot07</t>
-        </is>
+      <c r="A525" s="21" t="n">
+        <v>7</v>
       </c>
       <c r="B525" s="21" t="inlineStr">
         <is>
-          <t>null</t>
+          <t>Plan Görünümü</t>
         </is>
       </c>
       <c r="C525" s="21" t="inlineStr">
         <is>
-          <t>null</t>
+          <t>clip</t>
         </is>
       </c>
       <c r="D525" s="21" t="inlineStr">
         <is>
-          <t>null</t>
+          <t>CLIP_MODE</t>
         </is>
       </c>
       <c r="E525" s="21" t="inlineStr">
         <is>
-          <t>null</t>
+          <t>toggle-2</t>
         </is>
       </c>
       <c r="F525" s="21" t="n"/>
@@ -26891,7 +26889,7 @@
       <c r="G533" s="19" t="n"/>
       <c r="H533" s="19" t="inlineStr">
         <is>
-          <t>toggle-1-left</t>
+          <t>cam1-left</t>
         </is>
       </c>
       <c r="I533" s="19" t="n"/>
@@ -26928,7 +26926,7 @@
       <c r="G534" s="19" t="n"/>
       <c r="H534" s="19" t="inlineStr">
         <is>
-          <t>toggle-1-right</t>
+          <t>cam1-right</t>
         </is>
       </c>
       <c r="I534" s="19" t="n"/>
@@ -26965,7 +26963,7 @@
       <c r="G535" s="19" t="n"/>
       <c r="H535" s="19" t="inlineStr">
         <is>
-          <t>toggle-2-left</t>
+          <t>cam2-left</t>
         </is>
       </c>
       <c r="I535" s="19" t="n"/>
@@ -27001,7 +26999,7 @@
       <c r="G536" s="19" t="n"/>
       <c r="H536" s="19" t="inlineStr">
         <is>
-          <t>toggle-2-right</t>
+          <t>cam2-right</t>
         </is>
       </c>
       <c r="I536" s="19" t="n"/>
@@ -27038,7 +27036,7 @@
       <c r="G537" s="19" t="n"/>
       <c r="H537" s="19" t="inlineStr">
         <is>
-          <t>toggle-3-left</t>
+          <t>cam3-left</t>
         </is>
       </c>
       <c r="I537" s="19" t="n"/>
@@ -27074,7 +27072,7 @@
       <c r="G538" s="19" t="n"/>
       <c r="H538" s="19" t="inlineStr">
         <is>
-          <t>toggle-3-right</t>
+          <t>cam3-right</t>
         </is>
       </c>
       <c r="I538" s="19" t="n"/>
@@ -27111,7 +27109,7 @@
       <c r="G539" s="19" t="n"/>
       <c r="H539" s="19" t="inlineStr">
         <is>
-          <t>toggle-4-left</t>
+          <t>cam4-left</t>
         </is>
       </c>
       <c r="I539" s="19" t="n"/>
@@ -27147,7 +27145,7 @@
       <c r="G540" s="19" t="n"/>
       <c r="H540" s="19" t="inlineStr">
         <is>
-          <t>toggle-4-right</t>
+          <t>cam4-right</t>
         </is>
       </c>
       <c r="I540" s="19" t="n"/>
@@ -27182,7 +27180,7 @@
       <c r="G541" s="19" t="n"/>
       <c r="H541" s="19" t="inlineStr">
         <is>
-          <t>toggle-5-left</t>
+          <t>cam5-left</t>
         </is>
       </c>
       <c r="I541" s="19" t="n"/>
@@ -27217,7 +27215,7 @@
       <c r="G542" s="19" t="n"/>
       <c r="H542" s="19" t="inlineStr">
         <is>
-          <t>toggle-5-right</t>
+          <t>cam5-right</t>
         </is>
       </c>
       <c r="I542" s="19" t="n"/>
@@ -27253,7 +27251,7 @@
       <c r="G543" s="19" t="n"/>
       <c r="H543" s="19" t="inlineStr">
         <is>
-          <t>toggle-6-left</t>
+          <t>cam6-left</t>
         </is>
       </c>
       <c r="I543" s="19" t="n"/>
@@ -27289,7 +27287,7 @@
       <c r="G544" s="19" t="n"/>
       <c r="H544" s="19" t="inlineStr">
         <is>
-          <t>toggle-6-right</t>
+          <t>cam6-right</t>
         </is>
       </c>
       <c r="I544" s="19" t="n"/>
@@ -28310,439 +28308,325 @@
       </c>
     </row>
     <row r="567">
-      <c r="A567" s="21" t="inlineStr">
-        <is>
-          <t>slot01</t>
-        </is>
+      <c r="A567" s="21" t="n">
+        <v>1</v>
       </c>
       <c r="B567" s="21" t="inlineStr">
         <is>
-          <t>null</t>
+          <t>Salon
+32 m²</t>
         </is>
       </c>
       <c r="C567" s="21" t="inlineStr">
         <is>
-          <t>null</t>
-        </is>
-      </c>
-      <c r="D567" s="21" t="inlineStr">
-        <is>
-          <t>null</t>
-        </is>
-      </c>
+          <t>png</t>
+        </is>
+      </c>
+      <c r="D567" s="21" t="n"/>
       <c r="E567" s="21" t="inlineStr">
         <is>
-          <t>null</t>
+          <t>text</t>
         </is>
       </c>
       <c r="F567" s="21" t="inlineStr">
         <is>
-          <t>null</t>
-        </is>
-      </c>
-      <c r="G567" s="21" t="inlineStr">
-        <is>
-          <t>null</t>
-        </is>
-      </c>
-      <c r="H567" s="21" t="inlineStr">
-        <is>
-          <t>null</t>
-        </is>
-      </c>
-      <c r="I567" s="21" t="inlineStr">
-        <is>
-          <t>null</t>
-        </is>
-      </c>
-      <c r="J567" s="21" t="inlineStr">
-        <is>
-          <t>null</t>
-        </is>
-      </c>
-      <c r="K567" s="21" t="inlineStr">
-        <is>
-          <t>null</t>
-        </is>
-      </c>
-      <c r="L567" s="21" t="inlineStr">
-        <is>
-          <t>null</t>
-        </is>
-      </c>
-      <c r="M567" s="21" t="inlineStr">
-        <is>
-          <t>null</t>
-        </is>
+          <t>32 m²</t>
+        </is>
+      </c>
+      <c r="G567" s="21" t="n">
+        <v>1</v>
+      </c>
+      <c r="H567" s="21" t="n">
+        <v>1</v>
+      </c>
+      <c r="I567" s="21" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="J567" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="K567" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="L567" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="M567" s="21" t="n">
+        <v>1</v>
       </c>
       <c r="N567" s="21" t="inlineStr">
         <is>
-          <t>null</t>
+          <t>toggle-2</t>
         </is>
       </c>
       <c r="O567" s="21" t="n"/>
     </row>
     <row r="568">
-      <c r="A568" s="21" t="inlineStr">
-        <is>
-          <t>slot02</t>
-        </is>
+      <c r="A568" s="21" t="n">
+        <v>2</v>
       </c>
       <c r="B568" s="21" t="inlineStr">
         <is>
-          <t>null</t>
+          <t>Mutfak
+16 m²</t>
         </is>
       </c>
       <c r="C568" s="21" t="inlineStr">
         <is>
-          <t>null</t>
-        </is>
-      </c>
-      <c r="D568" s="21" t="inlineStr">
-        <is>
-          <t>null</t>
-        </is>
-      </c>
+          <t>png</t>
+        </is>
+      </c>
+      <c r="D568" s="21" t="n"/>
       <c r="E568" s="21" t="inlineStr">
         <is>
-          <t>null</t>
+          <t>text</t>
         </is>
       </c>
       <c r="F568" s="21" t="inlineStr">
         <is>
-          <t>null</t>
-        </is>
-      </c>
-      <c r="G568" s="21" t="inlineStr">
-        <is>
-          <t>null</t>
-        </is>
-      </c>
-      <c r="H568" s="21" t="inlineStr">
-        <is>
-          <t>null</t>
-        </is>
-      </c>
-      <c r="I568" s="21" t="inlineStr">
-        <is>
-          <t>null</t>
-        </is>
-      </c>
-      <c r="J568" s="21" t="inlineStr">
-        <is>
-          <t>null</t>
-        </is>
-      </c>
-      <c r="K568" s="21" t="inlineStr">
-        <is>
-          <t>null</t>
-        </is>
-      </c>
-      <c r="L568" s="21" t="inlineStr">
-        <is>
-          <t>null</t>
-        </is>
-      </c>
-      <c r="M568" s="21" t="inlineStr">
-        <is>
-          <t>null</t>
-        </is>
+          <t>16 m²</t>
+        </is>
+      </c>
+      <c r="G568" s="21" t="n">
+        <v>-2</v>
+      </c>
+      <c r="H568" s="21" t="n">
+        <v>1</v>
+      </c>
+      <c r="I568" s="21" t="n">
+        <v>3.1</v>
+      </c>
+      <c r="J568" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="K568" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="L568" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="M568" s="21" t="n">
+        <v>1</v>
       </c>
       <c r="N568" s="21" t="inlineStr">
         <is>
-          <t>null</t>
+          <t>toggle-2</t>
         </is>
       </c>
       <c r="O568" s="21" t="n"/>
     </row>
     <row r="569">
-      <c r="A569" s="21" t="inlineStr">
-        <is>
-          <t>slot03</t>
-        </is>
+      <c r="A569" s="21" t="n">
+        <v>3</v>
       </c>
       <c r="B569" s="21" t="inlineStr">
         <is>
-          <t>null</t>
+          <t>Bedroom 1
+18 m²</t>
         </is>
       </c>
       <c r="C569" s="21" t="inlineStr">
         <is>
-          <t>null</t>
-        </is>
-      </c>
-      <c r="D569" s="21" t="inlineStr">
-        <is>
-          <t>null</t>
-        </is>
-      </c>
+          <t>png</t>
+        </is>
+      </c>
+      <c r="D569" s="21" t="n"/>
       <c r="E569" s="21" t="inlineStr">
         <is>
-          <t>null</t>
+          <t>text</t>
         </is>
       </c>
       <c r="F569" s="21" t="inlineStr">
         <is>
-          <t>null</t>
-        </is>
-      </c>
-      <c r="G569" s="21" t="inlineStr">
-        <is>
-          <t>null</t>
-        </is>
-      </c>
-      <c r="H569" s="21" t="inlineStr">
-        <is>
-          <t>null</t>
-        </is>
-      </c>
-      <c r="I569" s="21" t="inlineStr">
-        <is>
-          <t>null</t>
-        </is>
-      </c>
-      <c r="J569" s="21" t="inlineStr">
-        <is>
-          <t>null</t>
-        </is>
-      </c>
-      <c r="K569" s="21" t="inlineStr">
-        <is>
-          <t>null</t>
-        </is>
-      </c>
-      <c r="L569" s="21" t="inlineStr">
-        <is>
-          <t>null</t>
-        </is>
-      </c>
-      <c r="M569" s="21" t="inlineStr">
-        <is>
-          <t>null</t>
-        </is>
+          <t>18 m²</t>
+        </is>
+      </c>
+      <c r="G569" s="21" t="n">
+        <v>-2</v>
+      </c>
+      <c r="H569" s="21" t="n">
+        <v>1</v>
+      </c>
+      <c r="I569" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="J569" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="K569" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="L569" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="M569" s="21" t="n">
+        <v>1</v>
       </c>
       <c r="N569" s="21" t="inlineStr">
         <is>
-          <t>null</t>
+          <t>toggle-2</t>
         </is>
       </c>
       <c r="O569" s="21" t="n"/>
     </row>
     <row r="570">
-      <c r="A570" s="21" t="inlineStr">
-        <is>
-          <t>slot04</t>
-        </is>
+      <c r="A570" s="21" t="n">
+        <v>4</v>
       </c>
       <c r="B570" s="21" t="inlineStr">
         <is>
-          <t>null</t>
+          <t>Bed 1 WC
+8 m²</t>
         </is>
       </c>
       <c r="C570" s="21" t="inlineStr">
         <is>
-          <t>null</t>
-        </is>
-      </c>
-      <c r="D570" s="21" t="inlineStr">
-        <is>
-          <t>null</t>
-        </is>
-      </c>
+          <t>png</t>
+        </is>
+      </c>
+      <c r="D570" s="21" t="n"/>
       <c r="E570" s="21" t="inlineStr">
         <is>
-          <t>null</t>
+          <t>text</t>
         </is>
       </c>
       <c r="F570" s="21" t="inlineStr">
         <is>
-          <t>null</t>
-        </is>
-      </c>
-      <c r="G570" s="21" t="inlineStr">
-        <is>
-          <t>null</t>
-        </is>
-      </c>
-      <c r="H570" s="21" t="inlineStr">
-        <is>
-          <t>null</t>
-        </is>
-      </c>
-      <c r="I570" s="21" t="inlineStr">
-        <is>
-          <t>null</t>
-        </is>
-      </c>
-      <c r="J570" s="21" t="inlineStr">
-        <is>
-          <t>null</t>
-        </is>
-      </c>
-      <c r="K570" s="21" t="inlineStr">
-        <is>
-          <t>null</t>
-        </is>
-      </c>
-      <c r="L570" s="21" t="inlineStr">
-        <is>
-          <t>null</t>
-        </is>
-      </c>
-      <c r="M570" s="21" t="inlineStr">
-        <is>
-          <t>null</t>
-        </is>
+          <t>8 m²</t>
+        </is>
+      </c>
+      <c r="G570" s="21" t="n">
+        <v>-2</v>
+      </c>
+      <c r="H570" s="21" t="n">
+        <v>1</v>
+      </c>
+      <c r="I570" s="21" t="n">
+        <v>2.1</v>
+      </c>
+      <c r="J570" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="K570" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="L570" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="M570" s="21" t="n">
+        <v>1</v>
       </c>
       <c r="N570" s="21" t="inlineStr">
         <is>
-          <t>null</t>
+          <t>toggle-2</t>
         </is>
       </c>
       <c r="O570" s="21" t="n"/>
     </row>
     <row r="571">
-      <c r="A571" s="21" t="inlineStr">
-        <is>
-          <t>slot05</t>
-        </is>
+      <c r="A571" s="21" t="n">
+        <v>5</v>
       </c>
       <c r="B571" s="21" t="inlineStr">
         <is>
-          <t>null</t>
+          <t>Bedroom 2
+14 m²</t>
         </is>
       </c>
       <c r="C571" s="21" t="inlineStr">
         <is>
-          <t>null</t>
-        </is>
-      </c>
-      <c r="D571" s="21" t="inlineStr">
-        <is>
-          <t>null</t>
-        </is>
-      </c>
+          <t>png</t>
+        </is>
+      </c>
+      <c r="D571" s="21" t="n"/>
       <c r="E571" s="21" t="inlineStr">
         <is>
-          <t>null</t>
+          <t>text</t>
         </is>
       </c>
       <c r="F571" s="21" t="inlineStr">
         <is>
-          <t>null</t>
-        </is>
-      </c>
-      <c r="G571" s="21" t="inlineStr">
-        <is>
-          <t>null</t>
-        </is>
-      </c>
-      <c r="H571" s="21" t="inlineStr">
-        <is>
-          <t>null</t>
-        </is>
-      </c>
-      <c r="I571" s="21" t="inlineStr">
-        <is>
-          <t>null</t>
-        </is>
-      </c>
-      <c r="J571" s="21" t="inlineStr">
-        <is>
-          <t>null</t>
-        </is>
-      </c>
-      <c r="K571" s="21" t="inlineStr">
-        <is>
-          <t>null</t>
-        </is>
-      </c>
-      <c r="L571" s="21" t="inlineStr">
-        <is>
-          <t>null</t>
-        </is>
-      </c>
-      <c r="M571" s="21" t="inlineStr">
-        <is>
-          <t>null</t>
-        </is>
+          <t>14 m²</t>
+        </is>
+      </c>
+      <c r="G571" s="21" t="n">
+        <v>4.4</v>
+      </c>
+      <c r="H571" s="21" t="n">
+        <v>1</v>
+      </c>
+      <c r="I571" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="J571" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="K571" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="L571" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="M571" s="21" t="n">
+        <v>1</v>
       </c>
       <c r="N571" s="21" t="inlineStr">
         <is>
-          <t>null</t>
+          <t>toggle-2</t>
         </is>
       </c>
       <c r="O571" s="21" t="n"/>
     </row>
     <row r="572">
-      <c r="A572" s="21" t="inlineStr">
-        <is>
-          <t>slot06</t>
-        </is>
+      <c r="A572" s="21" t="n">
+        <v>6</v>
       </c>
       <c r="B572" s="21" t="inlineStr">
         <is>
-          <t>null</t>
+          <t>Bed 2 WC
+5 m²</t>
         </is>
       </c>
       <c r="C572" s="21" t="inlineStr">
         <is>
-          <t>null</t>
-        </is>
-      </c>
-      <c r="D572" s="21" t="inlineStr">
-        <is>
-          <t>null</t>
-        </is>
-      </c>
+          <t>png</t>
+        </is>
+      </c>
+      <c r="D572" s="21" t="n"/>
       <c r="E572" s="21" t="inlineStr">
         <is>
-          <t>null</t>
+          <t>text</t>
         </is>
       </c>
       <c r="F572" s="21" t="inlineStr">
         <is>
-          <t>null</t>
-        </is>
-      </c>
-      <c r="G572" s="21" t="inlineStr">
-        <is>
-          <t>null</t>
-        </is>
-      </c>
-      <c r="H572" s="21" t="inlineStr">
-        <is>
-          <t>null</t>
-        </is>
-      </c>
-      <c r="I572" s="21" t="inlineStr">
-        <is>
-          <t>null</t>
-        </is>
-      </c>
-      <c r="J572" s="21" t="inlineStr">
-        <is>
-          <t>null</t>
-        </is>
-      </c>
-      <c r="K572" s="21" t="inlineStr">
-        <is>
-          <t>null</t>
-        </is>
-      </c>
-      <c r="L572" s="21" t="inlineStr">
-        <is>
-          <t>null</t>
-        </is>
-      </c>
-      <c r="M572" s="21" t="inlineStr">
-        <is>
-          <t>null</t>
-        </is>
+          <t>5 m²</t>
+        </is>
+      </c>
+      <c r="G572" s="21" t="n">
+        <v>3.9</v>
+      </c>
+      <c r="H572" s="21" t="n">
+        <v>1</v>
+      </c>
+      <c r="I572" s="21" t="n">
+        <v>3.7</v>
+      </c>
+      <c r="J572" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="K572" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="L572" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="M572" s="21" t="n">
+        <v>1</v>
       </c>
       <c r="N572" s="21" t="inlineStr">
         <is>
-          <t>null</t>
+          <t>toggle-2</t>
         </is>
       </c>
       <c r="O572" s="21" t="n"/>

</xml_diff>

<commit_message>
feat: data-driven teleport popup type (popupTip=teleport)
Teleport is now an Excel-defined popup type. Hotspots with
popupTip="teleport" show a toggle-switching teleport button
instead of regular content. Scene provides onTeleport callback
to handle the actual navigation.

- Added "teleport" to KNOWN_TIPS in xlsx-loader-4.js
- Updated 6 plan-view hotspots in Excel: popupTip=teleport
- _showPopup renders teleport UI only when data says so

https://claude.ai/code/session_01NbLjFLHf9cNBKyb3QMv6fy
</commit_message>
<xml_diff>
--- a/demo2-xlsx/demo2-input_4.xlsx
+++ b/demo2-xlsx/demo2-input_4.xlsx
@@ -28325,7 +28325,7 @@
       <c r="D567" s="21" t="n"/>
       <c r="E567" s="21" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>teleport</t>
         </is>
       </c>
       <c r="F567" s="21" t="inlineStr">
@@ -28379,7 +28379,7 @@
       <c r="D568" s="21" t="n"/>
       <c r="E568" s="21" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>teleport</t>
         </is>
       </c>
       <c r="F568" s="21" t="inlineStr">
@@ -28433,7 +28433,7 @@
       <c r="D569" s="21" t="n"/>
       <c r="E569" s="21" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>teleport</t>
         </is>
       </c>
       <c r="F569" s="21" t="inlineStr">
@@ -28487,7 +28487,7 @@
       <c r="D570" s="21" t="n"/>
       <c r="E570" s="21" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>teleport</t>
         </is>
       </c>
       <c r="F570" s="21" t="inlineStr">
@@ -28541,7 +28541,7 @@
       <c r="D571" s="21" t="n"/>
       <c r="E571" s="21" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>teleport</t>
         </is>
       </c>
       <c r="F571" s="21" t="inlineStr">
@@ -28595,7 +28595,7 @@
       <c r="D572" s="21" t="n"/>
       <c r="E572" s="21" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>teleport</t>
         </is>
       </c>
       <c r="F572" s="21" t="inlineStr">

</xml_diff>

<commit_message>
feat: configurable nav dot positions via Excel (Dot X/Y/Z)
Button rows now support optional columns F/G/H (Dot X, Dot Y, Dot Z).
If all three are filled, the floor teleport dot uses those coords
instead of the camera position. If empty, falls back to camera pos.

https://claude.ai/code/session_01NbLjFLHf9cNBKyb3QMv6fy
</commit_message>
<xml_diff>
--- a/demo2-xlsx/demo2-input_4.xlsx
+++ b/demo2-xlsx/demo2-input_4.xlsx
@@ -26409,6 +26409,21 @@
           <t>Kod</t>
         </is>
       </c>
+      <c r="F518" t="inlineStr">
+        <is>
+          <t>Dot X</t>
+        </is>
+      </c>
+      <c r="G518" t="inlineStr">
+        <is>
+          <t>Dot Y</t>
+        </is>
+      </c>
+      <c r="H518" t="inlineStr">
+        <is>
+          <t>Dot Z</t>
+        </is>
+      </c>
     </row>
     <row r="519">
       <c r="A519" s="19" t="n">

</xml_diff>